<commit_message>
fix(cdn & data): upload 31 CDN assets & sync Japan game boxarts and databases
</commit_message>
<xml_diff>
--- a/data/RetroVault_GS_Games_全量匯入檔.xlsx
+++ b/data/RetroVault_GS_Games_全量匯入檔.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RetroVault_Games" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Games" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -71126,11 +71126,19 @@
       </c>
       <c r="AH327" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/libretro-thumbnails/Nintendo_-_Game_Boy/master/Named_Boxarts/Quarth%20%28Japan%29.png</t>
-        </is>
-      </c>
-      <c r="AI327" t="inlineStr"/>
-      <c r="AJ327" t="inlineStr"/>
+          <t>https://raw.githubusercontent.com/Kevinte67228/Retro-library/main/docs/cdn/gb_quarth_jp_front.jpg</t>
+        </is>
+      </c>
+      <c r="AI327" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Kevinte67228/Retro-library/main/docs/cdn/gb_quarth_jp_back.jpg</t>
+        </is>
+      </c>
+      <c r="AJ327" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Kevinte67228/Retro-library/main/docs/cdn/gb_quarth_jp_spine.jpg</t>
+        </is>
+      </c>
       <c r="AK327" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/libretro-thumbnails/Nintendo_-_Game_Boy/master/Named_Snaps/Quarth%20%28Japan%29.png</t>
@@ -71337,11 +71345,19 @@
       </c>
       <c r="AH328" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/libretro-thumbnails/Nintendo_-_Game_Boy/master/Named_Boxarts/Hokuto%20no%20Ken%20-%20Seizetsu%20Juuban%20Shoubu%20%28Japan%29.png</t>
-        </is>
-      </c>
-      <c r="AI328" t="inlineStr"/>
-      <c r="AJ328" t="inlineStr"/>
+          <t>https://raw.githubusercontent.com/Kevinte67228/Retro-library/main/docs/cdn/gb_hokuto_jp_front.jpg</t>
+        </is>
+      </c>
+      <c r="AI328" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Kevinte67228/Retro-library/main/docs/cdn/gb_hokuto_jp_back.jpg</t>
+        </is>
+      </c>
+      <c r="AJ328" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Kevinte67228/Retro-library/main/docs/cdn/gb_hokuto_jp_spine.jpg</t>
+        </is>
+      </c>
       <c r="AK328" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/libretro-thumbnails/Nintendo_-_Game_Boy/master/Named_Snaps/Hokuto%20no%20Ken%20-%20Seizetsu%20Juuban%20Shoubu%20%28Japan%29.png</t>
@@ -71759,10 +71775,14 @@
       </c>
       <c r="AH330" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/libretro-thumbnails/Nintendo_-_Game_Boy/master/Named_Boxarts/Nekketsu%20Koukou%20Soccer-bu%20-%20World%20Cup%20Hen%20%28Japan%29.png</t>
-        </is>
-      </c>
-      <c r="AI330" t="inlineStr"/>
+          <t>https://raw.githubusercontent.com/Kevinte67228/Retro-library/main/docs/cdn/gb_nekketsu_soccer_jp_front.jpg</t>
+        </is>
+      </c>
+      <c r="AI330" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Kevinte67228/Retro-library/main/docs/cdn/gb_nekketsu_soccer_jp_back.jpg</t>
+        </is>
+      </c>
       <c r="AJ330" t="inlineStr"/>
       <c r="AK330" t="inlineStr">
         <is>
@@ -71970,11 +71990,19 @@
       </c>
       <c r="AH331" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/libretro-thumbnails/Nintendo_-_Game_Boy/master/Named_Boxarts/Nobunaga%20no%20Yabou%20-%20Game%20Boy%20Ban%20%28Japan%29.png</t>
-        </is>
-      </c>
-      <c r="AI331" t="inlineStr"/>
-      <c r="AJ331" t="inlineStr"/>
+          <t>https://raw.githubusercontent.com/Kevinte67228/Retro-library/main/docs/cdn/gb_nobunaga_jp_front.jpg</t>
+        </is>
+      </c>
+      <c r="AI331" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Kevinte67228/Retro-library/main/docs/cdn/gb_nobunaga_jp_back.jpg</t>
+        </is>
+      </c>
+      <c r="AJ331" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Kevinte67228/Retro-library/main/docs/cdn/gb_nobunaga_jp_spine.jpg</t>
+        </is>
+      </c>
       <c r="AK331" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/libretro-thumbnails/Nintendo_-_Game_Boy/master/Named_Snaps/Nobunaga%20no%20Yabou%20-%20Game%20Boy%20Ban%20%28Japan%29.png</t>
@@ -72603,10 +72631,14 @@
       </c>
       <c r="AH334" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/libretro-thumbnails/Nintendo_-_Game_Boy/master/Named_Boxarts/Boxing%20%28Japan%29.png</t>
-        </is>
-      </c>
-      <c r="AI334" t="inlineStr"/>
+          <t>https://raw.githubusercontent.com/Kevinte67228/Retro-library/main/docs/cdn/gb_boxing_jp_front.png</t>
+        </is>
+      </c>
+      <c r="AI334" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Kevinte67228/Retro-library/main/docs/cdn/gb_boxing_jp_back.jpg</t>
+        </is>
+      </c>
       <c r="AJ334" t="inlineStr"/>
       <c r="AK334" t="inlineStr">
         <is>
@@ -73244,11 +73276,19 @@
       </c>
       <c r="AH337" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/libretro-thumbnails/Nintendo_-_Game_Boy/master/Named_Boxarts/R-Type%20%28Japan%29.png</t>
-        </is>
-      </c>
-      <c r="AI337" t="inlineStr"/>
-      <c r="AJ337" t="inlineStr"/>
+          <t>https://raw.githubusercontent.com/Kevinte67228/Retro-library/main/docs/cdn/gb_rtype_jp_front.png</t>
+        </is>
+      </c>
+      <c r="AI337" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Kevinte67228/Retro-library/main/docs/cdn/gb_rtype_jp_back.png</t>
+        </is>
+      </c>
+      <c r="AJ337" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Kevinte67228/Retro-library/main/docs/cdn/gb_rtype_jp_spine.png</t>
+        </is>
+      </c>
       <c r="AK337" t="inlineStr">
         <is>
           <t>https://raw.githubusercontent.com/libretro-thumbnails/Nintendo_-_Game_Boy/master/Named_Snaps/R-Type%20%28Japan%29.png</t>
@@ -74096,14 +74136,14 @@
       </c>
       <c r="AH341" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/libretro-thumbnails/Sega_-_Game_Gear/master/Named_Boxarts/Sonic%20_%20Tails%202%20%28Japan%29%20%28En%29.png</t>
+          <t>https://raw.githubusercontent.com/Kevinte67228/Retro-library/main/docs/cdn/gg_sonic_tails_1_jp_front.png</t>
         </is>
       </c>
       <c r="AI341" t="inlineStr"/>
       <c r="AJ341" t="inlineStr"/>
       <c r="AK341" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/libretro-thumbnails/Sega_-_Game_Gear/master/Named_Snaps/Sonic%20_%20Tails%202%20%28Japan%29%20%28En%29.png</t>
+          <t>https://raw.githubusercontent.com/libretro-thumbnails/Sega_-_Game_Gear/master/Named_Snaps/Sonic%20_%20Tails%20(Japan)%20(En).png</t>
         </is>
       </c>
       <c r="AL341" t="inlineStr"/>
@@ -76918,22 +76958,22 @@
       </c>
       <c r="B355" t="inlineStr">
         <is>
-          <t>ピノビィの大冒険</t>
+          <t>ピノビィーの大冒険</t>
         </is>
       </c>
       <c r="C355" t="inlineStr">
         <is>
-          <t>ピノビィの大冒険</t>
+          <t>ピノビィーの大冒険</t>
         </is>
       </c>
       <c r="D355" t="inlineStr">
         <is>
-          <t>皮諾比大冒險</t>
+          <t>皮諾比的大冒險</t>
         </is>
       </c>
       <c r="E355" t="inlineStr">
         <is>
-          <t>Pinobee: Wings of Adventure</t>
+          <t>Pinobee: Quest of Heart</t>
         </is>
       </c>
       <c r="F355" t="inlineStr">
@@ -77058,7 +77098,7 @@
       </c>
       <c r="AH355" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/libretro-thumbnails/Nintendo_-_Game_Boy_Advance/master/Named_Boxarts/Pinobee%20no%20Daibouken%20%28Japan%29.png</t>
+          <t>https://raw.githubusercontent.com/Kevinte67228/Retro-library/main/docs/cdn/gba_pinobee_jp_front.jpg</t>
         </is>
       </c>
       <c r="AI355" t="inlineStr"/>
@@ -79588,7 +79628,11 @@
           <t>https://www.google.com/search?q=UP%20USB%20CARD%20256M%20Game%20Boy%20Advance</t>
         </is>
       </c>
-      <c r="AH367" t="inlineStr"/>
+      <c r="AH367" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Kevinte67228/Retro-library/main/docs/cdn/gba_up_usb_card_256m.jpg</t>
+        </is>
+      </c>
       <c r="AI367" t="inlineStr"/>
       <c r="AJ367" t="inlineStr"/>
       <c r="AK367" t="inlineStr"/>

</xml_diff>

<commit_message>
feat(assets & rules): add SFC reprint boxes, eliminate US SNES backs, and establish region integrity rules
</commit_message>
<xml_diff>
--- a/data/RetroVault_GS_Games_全量匯入檔.xlsx
+++ b/data/RetroVault_GS_Games_全量匯入檔.xlsx
@@ -8957,17 +8957,17 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>桃太郎活劇</t>
+          <t>桃太郎電鉄</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>桃太郎活劇</t>
+          <t>桃太郎電鉄</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>桃太郎活劇</t>
+          <t>桃太郎電鐵</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -36014,7 +36014,7 @@
       </c>
       <c r="AI164" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Kevinte67228/Retro-library/main/docs/cdn/7bd36c35-ba0e-4352-91a0-68184df3e5ee.jpg</t>
+          <t>https://raw.githubusercontent.com/Kevinte67228/Retro-library/main/docs/cdn/sfc_teitoku_jp_back.jpg</t>
         </is>
       </c>
       <c r="AJ164" t="inlineStr"/>
@@ -36227,11 +36227,7 @@
           <t>https://raw.githubusercontent.com/libretro-thumbnails/Nintendo_-_Super_Nintendo_Entertainment_System/master/Named_Boxarts/Teitoku%20no%20Ketsudan%20II%20%28Japan%29.png</t>
         </is>
       </c>
-      <c r="AI165" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/Kevinte67228/Retro-library/main/docs/cdn/76d52e61-4bb3-4e7f-bfc4-abc4cf49cb2a.jpg</t>
-        </is>
-      </c>
+      <c r="AI165" t="inlineStr"/>
       <c r="AJ165" t="inlineStr"/>
       <c r="AK165" t="inlineStr">
         <is>
@@ -36657,11 +36653,7 @@
           <t>https://raw.githubusercontent.com/libretro-thumbnails/Nintendo_-_Super_Nintendo_Entertainment_System/master/Named_Boxarts/Super%20Nobunaga%20no%20Yabou%20-%20Bushou%20Fuuunroku%20%28Japan%29.png</t>
         </is>
       </c>
-      <c r="AI167" t="inlineStr">
-        <is>
-          <t>https://raw.githubusercontent.com/Kevinte67228/Retro-library/main/docs/cdn/82d0864d-90f1-4f8a-abad-db3b25533533.jpg</t>
-        </is>
-      </c>
+      <c r="AI167" t="inlineStr"/>
       <c r="AJ167" t="inlineStr"/>
       <c r="AK167" t="inlineStr">
         <is>
@@ -36874,7 +36866,7 @@
       </c>
       <c r="AI168" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Kevinte67228/Retro-library/main/docs/cdn/eabf6d84-263e-4c7c-a063-daccfbfb1826.jpg</t>
+          <t>https://raw.githubusercontent.com/Kevinte67228/Retro-library/main/docs/cdn/sfc_kouryuuki_jp_back.jpg</t>
         </is>
       </c>
       <c r="AJ168" t="inlineStr"/>
@@ -42038,7 +42030,7 @@
       </c>
       <c r="AI192" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Kevinte67228/Retro-library/main/docs/cdn/857ba3b4-74e0-4879-aa2a-1a5638af1163.png</t>
+          <t>https://raw.githubusercontent.com/Kevinte67228/Retro-library/main/docs/cdn/sfc_bahamut_lagoon_jp_back.jpg</t>
         </is>
       </c>
       <c r="AJ192" t="inlineStr">
@@ -43117,7 +43109,7 @@
       </c>
       <c r="AI197" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Kevinte67228/Retro-library/main/docs/cdn/82d0864d-90f1-4f8a-abad-db3b25533533.jpg</t>
+          <t>https://raw.githubusercontent.com/Kevinte67228/Retro-library/main/docs/cdn/sfc_nobunaga_zenkoku_jp_back.jpg</t>
         </is>
       </c>
       <c r="AJ197" t="inlineStr"/>
@@ -44836,12 +44828,12 @@
       </c>
       <c r="AH205" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/libretro-thumbnails/Nintendo_-_Super_Nintendo_Entertainment_System/master/Named_Boxarts/Teitoku%20no%20Ketsudan%20%28Japan%29.png</t>
+          <t>https://raw.githubusercontent.com/Kevinte67228/Retro-library/main/docs/cdn/sfc_teitoku_reprint_jp_front.png</t>
         </is>
       </c>
       <c r="AI205" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Kevinte67228/Retro-library/main/docs/cdn/7bd36c35-ba0e-4352-91a0-68184df3e5ee.jpg</t>
+          <t>https://raw.githubusercontent.com/Kevinte67228/Retro-library/main/docs/cdn/sfc_teitoku_jp_back.jpg</t>
         </is>
       </c>
       <c r="AJ205" t="inlineStr"/>
@@ -45051,10 +45043,14 @@
       </c>
       <c r="AH206" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/libretro-thumbnails/Nintendo_-_Super_Nintendo_Entertainment_System/master/Named_Boxarts/Super%20Sangokushi%20II%20%28Japan%29.png</t>
-        </is>
-      </c>
-      <c r="AI206" t="inlineStr"/>
+          <t>https://raw.githubusercontent.com/Kevinte67228/Retro-library/main/docs/cdn/sfc_super_sangokushi2_reprint_jp_front.png</t>
+        </is>
+      </c>
+      <c r="AI206" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/Kevinte67228/Retro-library/main/docs/cdn/sfc_super_sangokushi2_reprint_jp_back.png</t>
+        </is>
+      </c>
       <c r="AJ206" t="inlineStr"/>
       <c r="AK206" t="inlineStr">
         <is>
@@ -53067,7 +53063,7 @@
       </c>
       <c r="AI243" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Kevinte67228/Retro-library/main/docs/cdn/6aebd916-c066-4c45-82a0-34378bd15990.png</t>
+          <t>https://raw.githubusercontent.com/Kevinte67228/Retro-library/main/docs/cdn/sfc_fe_monshou_jp_back.jpg</t>
         </is>
       </c>
       <c r="AJ243" t="inlineStr"/>
@@ -53282,7 +53278,7 @@
       </c>
       <c r="AI244" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Kevinte67228/Retro-library/main/docs/cdn/137b3f22-c980-4ee3-b9cd-b8a5ab10436f.png</t>
+          <t>https://raw.githubusercontent.com/Kevinte67228/Retro-library/main/docs/cdn/sfc_fe_seisen_jp_back.jpg</t>
         </is>
       </c>
       <c r="AJ244" t="inlineStr"/>
@@ -60413,7 +60409,7 @@
       </c>
       <c r="AI277" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Kevinte67228/Retro-library/main/docs/cdn/2906c1fc-0532-488e-af4c-c0e8d08b2012.jpg</t>
+          <t>https://raw.githubusercontent.com/Kevinte67228/Retro-library/main/docs/cdn/sfc_space_invaders_jp_back.jpg</t>
         </is>
       </c>
       <c r="AJ277" t="inlineStr">
@@ -64924,7 +64920,7 @@
       </c>
       <c r="AI298" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/Kevinte67228/Retro-library/main/docs/cdn/92109d5b-d550-40d8-8545-e5af8aea4d3f.jpg</t>
+          <t>https://raw.githubusercontent.com/Kevinte67228/Retro-library/main/docs/cdn/sfc_breath_of_fire_jp_back.jpg</t>
         </is>
       </c>
       <c r="AJ298" t="inlineStr">

</xml_diff>